<commit_message>
Technical Factor Engine + Observed/Used/Contribution factor snapshot
Adopt the user's key principle: never mix "available data" with "decision inputs".
- technical_factors.py: REAL indicators from OHLCV (EMAs, golden/death cross, RSI, ROC,
  momentum, rel-strength vs Nifty & Sector, ADX, realised vol, ATR%, Bollinger width,
  volume spike, OBV). Causal, not faked.
- Workbook "Factor Snapshot" sheet: every factor shown as Observed / Used by Strategy /
  Contribution. ONLY realised-vol + HRP + sector-cap + regime are Used=YES; all other
  technicals are Observed/Neutral; fundamentals/news = Not Evaluated (no data — not invented).
- Robust to the workbook being open in Excel (graceful fallback filename).

Honest scope: technical layer = built (we have OHLCV). Fundamental/earnings/news/institutional/
options layers stay Not Evaluated until that data is acquired (the Alpha Data Research roadmap).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/AEGIS_2026-06-25.xlsx
+++ b/reports/AEGIS_2026-06-25.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horizon Matrix" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical Performance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Why Picked" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Factor Snapshot" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registry" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
@@ -22861,7 +22861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:F145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22872,7 +22872,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Tier</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -22882,12 +22882,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Observed</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Used by Strategy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Contribution</t>
         </is>
       </c>
     </row>
@@ -22899,22 +22904,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>Above 20/50/100/200 EMA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>Yes/Yes/Yes/Yes</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -22926,22 +22936,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>50 vs 200 EMA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>12.7%</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -22953,22 +22968,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>RSI(14)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>56</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -22980,22 +23000,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>ROC(20)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>-0.3%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23007,22 +23032,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Momentum(10)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+8.6%</t>
+          <t>+1.0%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23034,22 +23064,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>Rel strength vs Nifty (3M)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>top 41%</t>
+          <t>+7.0%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23061,22 +23096,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>Rel strength vs Sector (3M)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>+4.6%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23088,22 +23128,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Trend strength</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>ADX(14)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23115,22 +23160,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Realised vol (20d, ann.)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
         </is>
       </c>
     </row>
@@ -23142,238 +23192,283 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>ATR(14) %</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>2.1%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>Bollinger band width</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>3.7%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>Volume spike (vs 20d)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>12.3%</t>
+          <t>0.8x</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>OBV trend</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>HRP cluster weight</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>12.7%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Sector cap &lt;= 2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+13.2%</t>
+          <t>diversified</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>Regime exposure</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>top 30%</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Fundamental</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>ROE/PE/EPS/Debt</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>MARICO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>News/Events</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>earnings/orders/upgrades</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>no data</t>
         </is>
       </c>
     </row>
@@ -23385,22 +23480,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Above 20/50/100/200 EMA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>Yes/Yes/Yes/Yes</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
@@ -23412,331 +23512,391 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>50 vs 200 EMA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>RSI(14)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>63</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>ROC(20)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>13.9%</t>
+          <t>+0.6%</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>Momentum(10)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>-0.8%</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>Rel strength vs Nifty (3M)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>+11.6%</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Rel strength vs Sector (3M)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>+2.4%</t>
+          <t>-2.5%</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Trend strength</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>ADX(14)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>top 58%</t>
+          <t>19</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>Realised vol (20d, ann.)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>ATR(14) %</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Bollinger band width</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>6.5%</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LUPIN</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>Volume spike (vs 20d)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>0.6x</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>OBV trend</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -23746,24 +23906,29 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>11.0%</t>
+          <t>12.3%</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -23778,19 +23943,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -23805,1249 +23975,3532 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Fundamental</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>ROE/PE/EPS/Debt</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>-10.9%</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>APOLLOHOSP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>News/Events</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>earnings/orders/upgrades</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>top 92%</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>no data</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>Above 20/50/100/200 EMA</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
+          <t>Yes/Yes/Yes/Yes</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>info</t>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>50 vs 200 EMA</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>RSI(14)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>69</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BRITANNIA</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>ROC(20)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>+3.1%</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>Momentum(10)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>+4.1%</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>Rel strength vs Nifty (3M)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>14.9%</t>
+          <t>+0.8%</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>Rel strength vs Sector (3M)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>-7.8%</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend strength</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>ADX(14)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Realised vol (20d, ann.)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>+2.5%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>ATR(14) %</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>top 57%</t>
+          <t>1.7%</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>Bollinger band width</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
+          <t>6.0%</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>info</t>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>Volume spike (vs 20d)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>0.9x</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>OBV trend</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BHARTIARTL</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>HRP cluster weight</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>13.9%</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>Sector cap &lt;= 2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>diversified</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>Regime exposure</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>10.4%</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Fundamental</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>ROE/PE/EPS/Debt</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>LUPIN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>News/Events</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>earnings/orders/upgrades</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>no data</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Above 20/50/100/200 EMA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>+0.1%</t>
+          <t>Yes/No/No/No</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>50 vs 200 EMA</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>top 66%</t>
+          <t>Death</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>RSI(14)</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>info</t>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>ROC(20)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>-1.6%</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Momentum(10)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>+2.6%</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ICICIGI</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>Rel strength vs Nifty (3M)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>-12.6%</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>Rel strength vs Sector (3M)</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>-15.0%</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend strength</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>ADX(14)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>13.6%</t>
+          <t>39</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>Realised vol (20d, ann.)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>ATR(14) %</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>1.4%</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volatility</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>Bollinger band width</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>-3.1%</t>
+          <t>6.0%</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>Volume spike (vs 20d)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>top 73%</t>
+          <t>0.6x</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Volume</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>OBV trend</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
+          <t>rising</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>info</t>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>HRP cluster weight</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>11.0%</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Portfolio</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Sector cap &lt;= 2</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>diversified</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ABBOTINDIA</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Macro</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>RSI / MACD / ADX</t>
+          <t>Regime exposure</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>not in model</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Positive</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Fundamental</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Low trailing volatility</t>
+          <t>ROE/PE/EPS/Debt</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>lowest-vol set</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>News/Events</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HRP cluster weight</t>
+          <t>earnings/orders/upgrades</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>11.2%</t>
+          <t>Not Evaluated</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>no data</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sector cap &lt;= 2</t>
+          <t>Above 20/50/100/200 EMA</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>diversified</t>
+          <t>Yes/Yes/Yes/Yes</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DRIVER</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Regime exposure</t>
+          <t>50 vs 200 EMA</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Death</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3M momentum</t>
+          <t>RSI(14)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>+3.8%</t>
+          <t>66</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Relative strength vs Nifty</t>
+          <t>ROC(20)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>top 53%</t>
+          <t>+1.4%</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>CONTEXT (not a driver)</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Above 200-DMA</t>
+          <t>Momentum(10)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
+          <t>+5.7%</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>info</t>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ROE / PE / EPS / Debt</t>
+          <t>Rel strength vs Nifty (3M)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
+          <t>+0.8%</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NOT EVALUATED</t>
+          <t>Momentum</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>News / earnings / events</t>
+          <t>Rel strength vs Sector (3M)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>no data</t>
+          <t>-7.0%</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Neutral</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Trend strength</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>ADX(14)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Realised vol (20d, ann.)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>17%</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ATR(14) %</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Bollinger band width</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>8.9%</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Volume spike (vs 20d)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>0.6x</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>OBV trend</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>rising</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>HRP cluster weight</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>14.9%</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Sector cap &lt;= 2</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>diversified</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Regime exposure</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Fundamental</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ROE/PE/EPS/Debt</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>News/Events</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>earnings/orders/upgrades</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>no data</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Above 20/50/100/200 EMA</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Yes/Yes/Yes/No</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>50 vs 200 EMA</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>RSI(14)</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ROC(20)</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>-1.1%</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Momentum(10)</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>+3.2%</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Rel strength vs Nifty (3M)</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>-1.5%</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Rel strength vs Sector (3M)</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>-5.4%</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Trend strength</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ADX(14)</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Realised vol (20d, ann.)</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>ATR(14) %</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Bollinger band width</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>12.3%</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Volume spike (vs 20d)</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>0.3x</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>OBV trend</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>rising</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>HRP cluster weight</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sector cap &lt;= 2</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>diversified</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Regime exposure</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Fundamental</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ROE/PE/EPS/Debt</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>News/Events</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>earnings/orders/upgrades</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>no data</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Above 20/50/100/200 EMA</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>No/No/No/No</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>50 vs 200 EMA</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>RSI(14)</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ROC(20)</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>-7.7%</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Momentum(10)</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>-2.0%</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Rel strength vs Nifty (3M)</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>-4.7%</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Rel strength vs Sector (3M)</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>-13.3%</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Trend strength</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>ADX(14)</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Realised vol (20d, ann.)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>19%</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>ATR(14) %</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>2.2%</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Bollinger band width</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>8.4%</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Volume spike (vs 20d)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>2.9x</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>OBV trend</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>falling</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>HRP cluster weight</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>13.6%</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sector cap &lt;= 2</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>diversified</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Regime exposure</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Fundamental</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ROE/PE/EPS/Debt</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>News/Events</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>earnings/orders/upgrades</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>no data</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
           <t>ICICIBANK</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>NOT EVALUATED</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>RSI / MACD / ADX</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>not in model</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Above 20/50/100/200 EMA</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Yes/Yes/Yes/Yes</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Trend</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>50 vs 200 EMA</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Death</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>RSI(14)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>ROC(20)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>+3.6%</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Momentum(10)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>+5.0%</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Rel strength vs Nifty (3M)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>+2.2%</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Momentum</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Rel strength vs Sector (3M)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>-1.7%</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Trend strength</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>ADX(14)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Realised vol (20d, ann.)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>18%</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Positive (low-vol = the driver)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ATR(14) %</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>1.9%</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Volatility</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Bollinger band width</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>13.3%</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Volume spike (vs 20d)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>0.7x</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Volume</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>OBV trend</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>rising</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>HRP cluster weight</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Sector cap &lt;= 2</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>diversified</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Regime exposure</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Fundamental</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>ROE/PE/EPS/Debt</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>no PIT data</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>News/Events</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>earnings/orders/upgrades</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Not Evaluated</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>no data</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Analytics: Portfolio Attribution + Stock Track Record + Yearly Quality + richer Statistics
The substantive (non-cosmetic) asks:
- Portfolio Attribution (the #1 missing piece): per stock, total/avg contribution across all
  historical cycles + times held + avg return. Shows what actually drove the cumulative result
  (top: IRFC +6.2, BHARTI +5.6; worst: RELAXO -3.8).
- Stock Track Record: times recommended, first/last, avg/best/worst return, win% per stock.
- Yearly Quality: per-year picks/winners/losers/win%/avg-return (2023 83%, 2022 53%, ...).
- Statistics: median winner/loser cycle, avg holding, avg drawdown-during-hold.

18 sheets. Held the line: still no fabricated fundamentals/forecasts; data-dependent layers
remain Not Evaluated. This is the end of Excel work per the review's own guidance.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/AEGIS_2026-06-25.xlsx
+++ b/reports/AEGIS_2026-06-25.xlsx
@@ -19,9 +19,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation Replay" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Strategy Replay" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation History" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Badges" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About AEGIS" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Portfolio Attribution" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock Track Record" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yearly Quality" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistics" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Badges" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About AEGIS" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26079,173 +26082,1383 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Times Held</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Total Contribution %</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Contribution %</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Return %</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Total cycles</t>
+          <t>IRFC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>19</v>
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6.19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16.75</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cycles beating Nifty</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>13 (68%)</t>
-        </is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5.61</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cycles positive</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>14 (74%)</t>
-        </is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="E4" t="n">
+        <v>24.57</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Avg portfolio return</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>+4.5%</t>
-        </is>
+          <t>MRF</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="E5" t="n">
+        <v>7.38</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Median portfolio return</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>+3.0%</t>
-        </is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>10.87</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Std deviation</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>6.4%</t>
-        </is>
+          <t>RVNL</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.19</v>
+      </c>
+      <c r="E7" t="n">
+        <v>101.25</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Avg outperformance vs Nifty</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>+2.1%</t>
-        </is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.67</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Best cycle</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>+14.8%</t>
-        </is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E9" t="n">
+        <v>13.24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Worst cycle</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>-6.4%</t>
-        </is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E10" t="n">
+        <v>24.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Avg winning cycle</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>+7.1%</t>
-        </is>
+          <t>LICI</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="E11" t="n">
+        <v>34.69</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Avg losing cycle</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>-2.8%</t>
-        </is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="E12" t="n">
+        <v>9.24</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Longest win streak</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>9 cycles</t>
-        </is>
+          <t>SUNDARMFIN</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="E13" t="n">
+        <v>24.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Longest loss streak</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>3 cycles</t>
-        </is>
+          <t>ALKEM</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="E14" t="n">
+        <v>8.199999999999999</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E16" t="n">
+        <v>11.08</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>BATAINDIA</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AIAENG</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E18" t="n">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="D19" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E19" t="n">
+        <v>30.95</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2.01</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.35</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>COLPAL</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.24</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="E22" t="n">
+        <v>4.13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E23" t="n">
+        <v>13.28</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>SUPREMEIND</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="E24" t="n">
+        <v>10.24</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PIIND</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="E25" t="n">
+        <v>18.91</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SJVN</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E26" t="n">
+        <v>11.66</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>10</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2.24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E29" t="n">
+        <v>8.94</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="D30" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="E30" t="n">
+        <v>25.86</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="E31" t="n">
+        <v>16.51</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="E32" t="n">
+        <v>7.73</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>VINATIORGA</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="E33" t="n">
+        <v>6.38</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>COROMANDEL</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E34" t="n">
+        <v>18.84</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3.82</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E37" t="n">
+        <v>8.06</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E38" t="n">
+        <v>12.33</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E39" t="n">
+        <v>9.029999999999999</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="E40" t="n">
+        <v>12.22</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E41" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>9</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.54</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E43" t="n">
+        <v>3.34</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>4</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>15</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SBICARD</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.94</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="E49" t="n">
+        <v>7.53</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="E50" t="n">
+        <v>7.84</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>PETRONET</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>3</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E51" t="n">
+        <v>2.71</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>3</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E52" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>NHPC</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E53" t="n">
+        <v>7.22</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>EXIDEIND</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="D54" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E54" t="n">
+        <v>4.59</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>7</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D55" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.52</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="D57" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>MGL</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="E58" t="n">
+        <v>-5.41</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-1.42</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ATUL</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>3</v>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="D60" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-3.46</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>IRCTC</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="D61" t="n">
+        <v>-0.47</v>
+      </c>
+      <c r="E61" t="n">
+        <v>-11.19</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>9</v>
+      </c>
+      <c r="C62" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="D62" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="D63" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="E63" t="n">
+        <v>-2.67</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>9</v>
+      </c>
+      <c r="C64" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="D64" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="E64" t="n">
+        <v>-1.25</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="D65" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="E65" t="n">
+        <v>-4.28</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>UBL</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>-0.79</v>
+      </c>
+      <c r="D66" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="E66" t="n">
+        <v>-7.03</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="D67" t="n">
+        <v>-0.44</v>
+      </c>
+      <c r="E67" t="n">
+        <v>-6.94</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n">
+        <v>-0.96</v>
+      </c>
+      <c r="D68" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="E68" t="n">
+        <v>-5.63</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="n">
+        <v>-0.99</v>
+      </c>
+      <c r="D69" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="E69" t="n">
+        <v>-9.43</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>15</v>
+      </c>
+      <c r="C70" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D70" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="E70" t="n">
+        <v>-0.75</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>RATNAMANI</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="D71" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="E71" t="n">
+        <v>-10.88</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>RELAXO</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" t="n">
+        <v>-3.82</v>
+      </c>
+      <c r="D72" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="E72" t="n">
+        <v>-10.85</v>
       </c>
     </row>
   </sheetData>
@@ -26259,126 +27472,2321 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Layer</t>
+          <t>Stock</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Times Recommended</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Detail</t>
+          <t>First</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Last</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Return %</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Best %</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Worst %</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Win %</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Portfolio Strategy</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>VALIDATED</t>
-        </is>
+          <t>TCS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>grade A · beat Nifty 68% of cycles</t>
-        </is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-16.6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Stock Selection (alpha)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>EXPERIMENTAL</t>
-        </is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RQS 0.51 ~ random · holdings, not bets</t>
-        </is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>53.3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Recommendation Horizon</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>HISTORICALLY TESTED</t>
-        </is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>13</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>all horizons backtested · best = 6M</t>
-        </is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>69.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Technical Context</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>COMPUTED (not a driver)</t>
-        </is>
+          <t>SUNPHARMA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>momentum / rel-strength / 200-DMA shown for info</t>
-        </is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F5" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-9.800000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>66.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fundamental Analysis</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>NOT EVALUATED</t>
-        </is>
+          <t>MRF</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>no point-in-time data</t>
-        </is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>News / Events</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>NOT EVALUATED</t>
-        </is>
+          <t>NESTLEIND</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>no event database</t>
-        </is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-8.4</v>
+      </c>
+      <c r="H7" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>22</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-23.8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>55.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F9" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-23.6</v>
+      </c>
+      <c r="H9" t="n">
+        <v>55.6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-16.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>55.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RELIANCE</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="H11" t="n">
+        <v>62.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="H12" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>COLPAL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2023-07-13</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-13.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="F14" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>85.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>DRREDDY</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-7.8</v>
+      </c>
+      <c r="H15" t="n">
+        <v>57.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ULTRACEMCO</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-12.9</v>
+      </c>
+      <c r="H16" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>INFY</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>14</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-19.8</v>
+      </c>
+      <c r="H17" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BAJAJ-AUTO</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>17.7</v>
+      </c>
+      <c r="G18" t="n">
+        <v>-14.9</v>
+      </c>
+      <c r="H18" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>-4.3</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BATAINDIA</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="F20" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="H20" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>9.699999999999999</v>
+      </c>
+      <c r="G21" t="n">
+        <v>-15.2</v>
+      </c>
+      <c r="H21" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ALKEM</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="F22" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G22" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="H22" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AIAENG</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="F23" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="G23" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="H23" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>APOLLOHOSP</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G24" t="n">
+        <v>-2.9</v>
+      </c>
+      <c r="H24" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GRASIM</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="F25" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TORNTPHARM</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F26" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="H26" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RELAXO</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>-10.8</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-26</v>
+      </c>
+      <c r="H27" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>HINDUNILVR</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2023-10-13</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="H28" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TITAN</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2023-10-13</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F29" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>NTPC</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ATUL</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="F31" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="G31" t="n">
+        <v>-12</v>
+      </c>
+      <c r="H31" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>HDFCLIFE</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>-5.6</v>
+      </c>
+      <c r="F32" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>-12.4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>SJVN</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>20.7</v>
+      </c>
+      <c r="G33" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="H33" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>EICHERMOT</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G34" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="H34" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>IRFC</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="F35" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-9.9</v>
+      </c>
+      <c r="H35" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>PETRONET</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F36" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="G36" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="H36" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>KOTAKBANK</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H37" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>COALINDIA</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2025-04-24</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G38" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="H38" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>BRITANNIA</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>-2.7</v>
+      </c>
+      <c r="F39" t="n">
+        <v>9</v>
+      </c>
+      <c r="G39" t="n">
+        <v>-9.300000000000001</v>
+      </c>
+      <c r="H39" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ACC</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="F40" t="n">
+        <v>-5.1</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2023-10-13</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F41" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="G41" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H41" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>VINATIORGA</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2024-04-18</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F42" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-4.9</v>
+      </c>
+      <c r="H42" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F43" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="G43" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H43" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>SUPREMEIND</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G44" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H44" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PFC</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="G45" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="H45" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UBL</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>-7</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>-16.5</v>
+      </c>
+      <c r="H46" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>POWERGRID</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F47" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="G47" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="H47" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SBICARD</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2024-10-18</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H48" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>ICICIGI</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F49" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G49" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="H49" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>HEROMOTOCO</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>-9.4</v>
+      </c>
+      <c r="F50" t="n">
+        <v>-5.8</v>
+      </c>
+      <c r="G50" t="n">
+        <v>-13</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>EXIDEIND</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F51" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="G51" t="n">
+        <v>-1.7</v>
+      </c>
+      <c r="H51" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MARICO</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F52" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="G52" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H52" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>IOC</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="G53" t="n">
+        <v>-2.6</v>
+      </c>
+      <c r="H53" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ONGC</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2025-10-24</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>9</v>
+      </c>
+      <c r="F54" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="G54" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="H54" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>RATNAMANI</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>-10.9</v>
+      </c>
+      <c r="F55" t="n">
+        <v>-9.699999999999999</v>
+      </c>
+      <c r="G55" t="n">
+        <v>-12.1</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>OFSS</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>16</v>
+      </c>
+      <c r="G56" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="H56" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>WIPRO</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>2023-07-13</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G57" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H57" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>IRCTC</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="F58" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="G58" t="n">
+        <v>-11.2</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="F59" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="G59" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="H59" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>BAJAJHLDNG</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>31</v>
+      </c>
+      <c r="F60" t="n">
+        <v>31</v>
+      </c>
+      <c r="G60" t="n">
+        <v>31</v>
+      </c>
+      <c r="H60" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CIPLA</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2025-07-23</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F61" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G61" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H61" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>CUMMINSIND</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>2022-07-06</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="F62" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G62" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="H62" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>COROMANDEL</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>2022-04-05</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="F63" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G63" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="H63" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>HCLTECH</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="F64" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G64" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H64" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>LICI</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2023-10-13</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>2023-10-13</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="F65" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="G65" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="H65" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>PIIND</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2024-07-19</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="F66" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="G66" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H66" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>NHPC</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="F67" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G67" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H67" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>MGL</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>2022-01-03</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="F68" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="G68" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>RVNL</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>2022-10-07</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="F69" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="G69" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="H69" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SBILIFE</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SUNDARMFIN</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2023-07-13</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>2023-07-13</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F71" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="G71" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="H71" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>TATACONSUM</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2023-04-12</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="F72" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="G72" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H72" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -26387,6 +29795,533 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Picks</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Winners</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Losers</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Win %</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Avg Return %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>63</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B3" t="n">
+        <v>60</v>
+      </c>
+      <c r="C3" t="n">
+        <v>32</v>
+      </c>
+      <c r="D3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" t="n">
+        <v>53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B4" t="n">
+        <v>60</v>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="n">
+        <v>83</v>
+      </c>
+      <c r="F4" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B5" t="n">
+        <v>60</v>
+      </c>
+      <c r="C5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D5" t="n">
+        <v>23</v>
+      </c>
+      <c r="E5" t="n">
+        <v>62</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B6" t="n">
+        <v>60</v>
+      </c>
+      <c r="C6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D6" t="n">
+        <v>25</v>
+      </c>
+      <c r="E6" t="n">
+        <v>58</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total cycles</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cycles beating Nifty</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>13 (68%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cycles positive</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>14 (74%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Avg portfolio return</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>+4.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Median portfolio return</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>+3.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Std deviation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Avg outperformance vs Nifty</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>+2.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Best cycle</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>+14.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Worst cycle</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>-6.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Avg winning cycle</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>+7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Avg losing cycle</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>-2.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Median winning cycle</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>+5.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Median losing cycle</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>-1.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Avg holding period</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6 months (63 trading days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Avg drawdown during hold</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>-5.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Longest win streak</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>9 cycles</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Longest loss streak</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3 cycles</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Layer</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Portfolio Strategy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VALIDATED</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>grade A · beat Nifty 68% of cycles</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Stock Selection (alpha)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EXPERIMENTAL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>RQS 0.51 ~ random · holdings, not bets</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Recommendation Horizon</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HISTORICALLY TESTED</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>all horizons backtested · best = 6M</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Technical Context</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>COMPUTED (not a driver)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>momentum / rel-strength / 200-DMA shown for info</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fundamental Analysis</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NOT EVALUATED</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>no point-in-time data</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>News / Events</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>NOT EVALUATED</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>no event database</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>